<commit_message>
Fix conversion script failures under StrictMode and empty export rows.
ConvertTo-ObjectArray now unwraps Generic.List safely, header arrays are no longer double-wrapped, and ImportExcel installs to a local Modules folder.
</commit_message>
<xml_diff>
--- a/sharepoint_list.xlsx
+++ b/sharepoint_list.xlsx
@@ -14,11 +14,12 @@
   </bookViews>
   <sheets>
     <sheet name="query (26)" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="query__26" localSheetId="0" hidden="1">'query (26)'!$A$1:$AK$3</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -31,11 +32,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>Title</t>
   </si>
   <si>
+    <t>EEmri</t>
+  </si>
+  <si>
     <t>DOB</t>
   </si>
   <si>
@@ -60,6 +64,9 @@
     <t>Lloji i punësimit</t>
   </si>
   <si>
+    <t>Statusi</t>
+  </si>
+  <si>
     <t>Projekti</t>
   </si>
   <si>
@@ -105,9 +112,6 @@
     <t>Comment</t>
   </si>
   <si>
-    <t>Statusi</t>
-  </si>
-  <si>
     <t>Data e përfundimit të Punës</t>
   </si>
   <si>
@@ -135,13 +139,13 @@
     <t xml:space="preserve">Pushime te tjera </t>
   </si>
   <si>
-    <t>EEmri</t>
+    <t>Item Type</t>
   </si>
   <si>
     <t>Path</t>
   </si>
   <si>
-    <t>Item Type</t>
+    <t>Andi Sokoli</t>
   </si>
   <si>
     <t>Mashkull</t>
@@ -150,49 +154,91 @@
     <t>Shqiptar</t>
   </si>
   <si>
+    <t>Mjekë</t>
+  </si>
+  <si>
     <t>Primar</t>
   </si>
   <si>
     <t>Active</t>
   </si>
   <si>
+    <t>PSH Viti</t>
+  </si>
+  <si>
+    <t>Viti</t>
+  </si>
+  <si>
+    <t>KO-09204-01</t>
+  </si>
+  <si>
+    <t>17020030325937-11</t>
+  </si>
+  <si>
+    <t>Doktor i Mjekesis</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
     <t>personal/bleona_ademi_caritaskosova_org/Lists/Lista e stafit 2026</t>
   </si>
   <si>
-    <t>Item</t>
+    <t>Rinë Krasniqi Musliu</t>
   </si>
   <si>
     <t>Femër</t>
   </si>
   <si>
-    <t>Viti</t>
-  </si>
-  <si>
-    <t>PSH Viti</t>
-  </si>
-  <si>
-    <t>Mjekë</t>
-  </si>
-  <si>
-    <t>Doktor i Mjekesis</t>
-  </si>
-  <si>
-    <t>Andi Sokoli</t>
-  </si>
-  <si>
-    <t>KO-09204-01</t>
-  </si>
-  <si>
-    <t>17020030325937-11</t>
-  </si>
-  <si>
-    <t>Rinë Krasniqi Musliu</t>
-  </si>
-  <si>
     <t>KO-07992-01</t>
   </si>
   <si>
     <t>19600093250211-50</t>
+  </si>
+  <si>
+    <t>Kualifikimi</t>
+  </si>
+  <si>
+    <t>Artan Krasniqi</t>
+  </si>
+  <si>
+    <t>artan.krasniqi@caritaskosova.org</t>
+  </si>
+  <si>
+    <t>IT Department</t>
+  </si>
+  <si>
+    <t>Developer</t>
+  </si>
+  <si>
+    <t>Senior</t>
+  </si>
+  <si>
+    <t>Prishtina</t>
+  </si>
+  <si>
+    <t>2020-01-15</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Bleona Ademi</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>HR Officer</t>
+  </si>
+  <si>
+    <t>Officer</t>
+  </si>
+  <si>
+    <t>2021-06-01</t>
+  </si>
+  <si>
+    <t>Jo aktiv</t>
   </si>
 </sst>
 </file>
@@ -202,7 +248,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-407]_-;\-* #,##0.00\ [$€-407]_-;_-* &quot;-&quot;??\ [$€-407]_-;_-@_-"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -637,100 +683,141 @@
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="46">
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="10" applyFill="1" borderId="0" applyBorder="1" xfId="1" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="14" applyFill="1" borderId="0" applyBorder="1" xfId="2" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="18" applyFill="1" borderId="0" applyBorder="1" xfId="3" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="22" applyFill="1" borderId="0" applyBorder="1" xfId="4" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="26" applyFill="1" borderId="0" applyBorder="1" xfId="5" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="30" applyFill="1" borderId="0" applyBorder="1" xfId="6" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="11" applyFill="1" borderId="0" applyBorder="1" xfId="7" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="15" applyFill="1" borderId="0" applyBorder="1" xfId="8" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="19" applyFill="1" borderId="0" applyBorder="1" xfId="9" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="23" applyFill="1" borderId="0" applyBorder="1" xfId="10" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="27" applyFill="1" borderId="0" applyBorder="1" xfId="11" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="31" applyFill="1" borderId="0" applyBorder="1" xfId="12" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="12" applyFill="1" borderId="0" applyBorder="1" xfId="13" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="16" applyFill="1" borderId="0" applyBorder="1" xfId="14" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="20" applyFill="1" borderId="0" applyBorder="1" xfId="15" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="24" applyFill="1" borderId="0" applyBorder="1" xfId="16" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="28" applyFill="1" borderId="0" applyBorder="1" xfId="17" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="32" applyFill="1" borderId="0" applyBorder="1" xfId="18" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="17" applyFont="1" fillId="9" applyFill="1" borderId="0" applyBorder="1" xfId="19" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="17" applyFont="1" fillId="13" applyFill="1" borderId="0" applyBorder="1" xfId="20" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="17" applyFont="1" fillId="17" applyFill="1" borderId="0" applyBorder="1" xfId="21" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="17" applyFont="1" fillId="21" applyFill="1" borderId="0" applyBorder="1" xfId="22" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="17" applyFont="1" fillId="25" applyFill="1" borderId="0" applyBorder="1" xfId="23" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="17" applyFont="1" fillId="29" applyFill="1" borderId="0" applyBorder="1" xfId="24" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="7" applyFont="1" fillId="3" applyFill="1" borderId="0" applyBorder="1" xfId="25" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="11" applyFont="1" fillId="6" applyFill="1" borderId="4" applyBorder="1" xfId="26" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="13" applyFont="1" fillId="7" applyFill="1" borderId="7" applyBorder="1" xfId="27" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="15" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="28" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="6" applyFont="1" fillId="2" applyFill="1" borderId="0" applyBorder="1" xfId="29" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="3" applyFont="1" fillId="0" applyFill="1" borderId="1" applyBorder="1" xfId="30" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="4" applyFont="1" fillId="0" applyFill="1" borderId="2" applyBorder="1" xfId="31" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="5" applyFont="1" fillId="0" applyFill="1" borderId="3" applyBorder="1" xfId="32" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="5" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="33" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="9" applyFont="1" fillId="5" applyFill="1" borderId="4" applyBorder="1" xfId="34" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="12" applyFont="1" fillId="0" applyFill="1" borderId="6" applyBorder="1" xfId="35" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="8" applyFont="1" fillId="4" applyFill="1" borderId="0" applyBorder="1" xfId="36" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="8" applyFill="1" borderId="8" applyBorder="1" xfId="37" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="10" applyFont="1" fillId="6" applyFill="1" borderId="5" applyBorder="1" xfId="38" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="39" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="16" applyFont="1" fillId="0" applyFill="1" borderId="9" applyBorder="1" xfId="40" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="14" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="41" applyProtection="1"/>
+    <xf numFmtId="49" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="14" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="1" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="2" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="3" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="4" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="5" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="6" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="7" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="8" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="9" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="10" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="11" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="12" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="13" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="14" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="15" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="16" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="17" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="18" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="19" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="20" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="21" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="22" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="23" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="24" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="25" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="26" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="27" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="28" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="29" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="30" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="31" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="32" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="33" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="34" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="35" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="36" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="37" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="38" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="39" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="40" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="41" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="37">
     <dxf>
@@ -1277,330 +1364,499 @@
   <dimension ref="A1:AK3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="81.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" bestFit="1" width="25.28515625" customWidth="1"/>
+    <col min="3" max="3" bestFit="1" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" bestFit="1" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="19" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="81.140625" customWidth="1"/>
+    <col min="8" max="8" bestFit="1" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" bestFit="1" width="36.85546875" customWidth="1"/>
+    <col min="10" max="10" bestFit="1" width="17.85546875" customWidth="1"/>
+    <col min="11" max="11" bestFit="1" width="9.5703125" customWidth="1"/>
     <col min="12" max="12" width="34.140625" customWidth="1"/>
-    <col min="13" max="13" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" bestFit="1" width="15.5703125" customWidth="1"/>
     <col min="14" max="14" width="31.5703125" customWidth="1"/>
-    <col min="15" max="15" width="29.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="32.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="81.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="29" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="31.7109375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="81.140625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="61.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" bestFit="1" width="29.85546875" customWidth="1"/>
+    <col min="16" max="16" bestFit="1" width="24.140625" customWidth="1"/>
+    <col min="17" max="17" bestFit="1" width="27.140625" customWidth="1"/>
+    <col min="18" max="18" bestFit="1" width="32.140625" customWidth="1"/>
+    <col min="19" max="19" bestFit="1" width="22" customWidth="1"/>
+    <col min="20" max="20" bestFit="1" width="12.7109375" customWidth="1"/>
+    <col min="21" max="21" bestFit="1" width="12.28515625" customWidth="1"/>
+    <col min="22" max="22" bestFit="1" width="44.85546875" customWidth="1"/>
+    <col min="23" max="24" bestFit="1" width="22.85546875" customWidth="1"/>
+    <col min="25" max="26" bestFit="1" width="81.140625" customWidth="1"/>
+    <col min="27" max="27" bestFit="1" width="29" customWidth="1"/>
+    <col min="28" max="28" bestFit="1" width="24.5703125" customWidth="1"/>
+    <col min="29" max="29" bestFit="1" width="24.140625" customWidth="1"/>
+    <col min="30" max="30" bestFit="1" width="26.28515625" customWidth="1"/>
+    <col min="31" max="31" bestFit="1" width="31.7109375" customWidth="1"/>
+    <col min="32" max="32" bestFit="1" width="19.7109375" customWidth="1"/>
+    <col min="33" max="33" bestFit="1" width="31.85546875" customWidth="1"/>
+    <col min="34" max="34" bestFit="1" width="24.28515625" customWidth="1"/>
+    <col min="35" max="35" bestFit="1" width="81.140625" customWidth="1"/>
+    <col min="36" max="36" bestFit="1" width="12.140625" customWidth="1"/>
+    <col min="37" max="37" bestFit="1" width="61.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" t="s">
-        <v>12</v>
-      </c>
-      <c r="P1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>14</v>
-      </c>
-      <c r="R1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S1" t="s">
-        <v>16</v>
-      </c>
-      <c r="T1" t="s">
-        <v>17</v>
-      </c>
-      <c r="U1" t="s">
-        <v>18</v>
-      </c>
-      <c r="V1" t="s">
-        <v>19</v>
-      </c>
-      <c r="W1" t="s">
-        <v>20</v>
-      </c>
-      <c r="X1" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="AK1" t="s">
-        <v>35</v>
-      </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2">
+      <c r="A2" s="42" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="42" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="43">
+        <v>36200</v>
+      </c>
+      <c r="D2" s="0">
+        <v>1172291291</v>
+      </c>
+      <c r="E2" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" s="44"/>
+      <c r="J2" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="K2" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="L2" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="M2" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" s="42" t="s">
+        <v>45</v>
+      </c>
+      <c r="O2" s="43">
+        <v>47918</v>
+      </c>
+      <c r="P2" s="43">
+        <v>46134</v>
+      </c>
+      <c r="Q2" s="43">
+        <v>46134</v>
+      </c>
+      <c r="R2" s="43">
+        <v>46387</v>
+      </c>
+      <c r="S2" s="42" t="s">
+        <v>46</v>
+      </c>
+      <c r="T2" s="45">
+        <v>650</v>
+      </c>
+      <c r="U2" s="45">
+        <v>558.29</v>
+      </c>
+      <c r="V2" s="44"/>
+      <c r="W2" s="44"/>
+      <c r="X2" s="44"/>
+      <c r="Y2" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z2" s="44"/>
+      <c r="AA2" s="43"/>
+      <c r="AB2" s="42"/>
+      <c r="AC2" s="43">
+        <v>46347</v>
+      </c>
+      <c r="AD2" s="43">
+        <v>46112</v>
+      </c>
+      <c r="AE2" s="42"/>
+      <c r="AF2" s="44"/>
+      <c r="AG2" s="44"/>
+      <c r="AH2" s="44"/>
+      <c r="AI2" s="44"/>
+      <c r="AJ2" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="AK2" s="42" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="42" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="43">
+        <v>34645</v>
+      </c>
+      <c r="D3" s="0">
+        <v>1230161018</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="44"/>
+      <c r="J3" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="K3" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="L3" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3" s="42" t="s">
+        <v>52</v>
+      </c>
+      <c r="O3" s="43">
+        <v>46450</v>
+      </c>
+      <c r="P3" s="43">
+        <v>46134</v>
+      </c>
+      <c r="Q3" s="43">
+        <v>46134</v>
+      </c>
+      <c r="R3" s="43">
+        <v>46387</v>
+      </c>
+      <c r="S3" s="42" t="s">
+        <v>53</v>
+      </c>
+      <c r="T3" s="45">
+        <v>650</v>
+      </c>
+      <c r="U3" s="45">
+        <v>558.29</v>
+      </c>
+      <c r="V3" s="44"/>
+      <c r="W3" s="44"/>
+      <c r="X3" s="44"/>
+      <c r="Y3" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z3" s="44"/>
+      <c r="AA3" s="43"/>
+      <c r="AB3" s="42"/>
+      <c r="AC3" s="43">
+        <v>48867</v>
+      </c>
+      <c r="AD3" s="43">
+        <v>46111</v>
+      </c>
+      <c r="AE3" s="42"/>
+      <c r="AF3" s="44"/>
+      <c r="AG3" s="44"/>
+      <c r="AH3" s="44"/>
+      <c r="AI3" s="44"/>
+      <c r="AJ3" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="2">
-        <v>36200</v>
-      </c>
-      <c r="D2">
-        <v>1172291291</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="N2" s="1" t="s">
+      <c r="AK3" s="42" t="s">
         <v>49</v>
-      </c>
-      <c r="O2" s="2">
-        <v>47918</v>
-      </c>
-      <c r="P2" s="2">
-        <v>46134</v>
-      </c>
-      <c r="Q2" s="2">
-        <v>46134</v>
-      </c>
-      <c r="R2" s="2">
-        <v>46387</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="T2" s="4">
-        <v>650</v>
-      </c>
-      <c r="U2" s="4">
-        <v>558.29</v>
-      </c>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-      <c r="Y2" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z2" s="3"/>
-      <c r="AA2" s="2"/>
-      <c r="AB2" s="1"/>
-      <c r="AC2" s="2">
-        <v>46347</v>
-      </c>
-      <c r="AD2" s="2">
-        <v>46112</v>
-      </c>
-      <c r="AE2" s="1"/>
-      <c r="AF2" s="3"/>
-      <c r="AG2" s="3"/>
-      <c r="AH2" s="3"/>
-      <c r="AI2" s="3"/>
-      <c r="AJ2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AK2" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="2">
-        <v>34645</v>
-      </c>
-      <c r="D3">
-        <v>1230161018</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="O3" s="2">
-        <v>46450</v>
-      </c>
-      <c r="P3" s="2">
-        <v>46134</v>
-      </c>
-      <c r="Q3" s="2">
-        <v>46134</v>
-      </c>
-      <c r="R3" s="2">
-        <v>46387</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="T3" s="4">
-        <v>650</v>
-      </c>
-      <c r="U3" s="4">
-        <v>558.29</v>
-      </c>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z3" s="3"/>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="1"/>
-      <c r="AC3" s="2">
-        <v>48867</v>
-      </c>
-      <c r="AD3" s="2">
-        <v>46111</v>
-      </c>
-      <c r="AE3" s="1"/>
-      <c r="AF3" s="3"/>
-      <c r="AG3" s="3"/>
-      <c r="AH3" s="3"/>
-      <c r="AI3" s="3"/>
-      <c r="AJ3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AK3" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10.9804048538208" customWidth="1"/>
+    <col min="2" max="2" width="14.9642210006714" customWidth="1"/>
+    <col min="3" max="3" width="13.4132537841797" customWidth="1"/>
+    <col min="4" max="4" width="33.5062599182129" customWidth="1"/>
+    <col min="5" max="5" width="14.6133098602295" customWidth="1"/>
+    <col min="6" max="6" width="9.9532470703125" customWidth="1"/>
+    <col min="7" max="7" width="15.1770181655884" customWidth="1"/>
+    <col min="8" max="8" width="15.6486520767212" customWidth="1"/>
+    <col min="9" max="9" width="11.1891098022461" customWidth="1"/>
+    <col min="10" max="10" width="16.1878070831299" customWidth="1"/>
+    <col min="11" max="11" width="14.7012939453125" customWidth="1"/>
+    <col min="12" max="12" width="22.5983333587646" customWidth="1"/>
+    <col min="13" max="13" width="12.182505607605" customWidth="1"/>
+    <col min="14" max="14" width="30.8370800018311" customWidth="1"/>
+    <col min="15" max="15" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="0">
+        <v>1234567890</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="0">
+        <v>38344123456</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="M2" s="0">
+        <v>850</v>
+      </c>
+      <c r="N2" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="O2" s="0" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="0">
+        <v>9876543210</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="0">
+        <v>44987654</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="J3" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="K3" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="L3" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="M3" s="0">
+        <v>700</v>
+      </c>
+      <c r="N3" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="O3" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>